<commit_message>
Kierunek Zysk: Dziennik decyzji i ścieżka do konsultacji Przegląd Decyzji (3 000 zł)
Nowy materiał 7 dla klienta (karty decyzji z tokiem rozumowania, 6 ogniw
jakości decyzji, pułapki myślenia, oferta i karta przygotowania), zaproszenia
w przewodniku, planerze i kalkulatorze (arkusz Podsumowanie), oraz pakiet
prowadzącej: maile po zakupie, kwalifikacja, analiza, scenariusz sesji,
karta analizy w Excelu z automatycznym raportem dla klienta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HrBtPyhm8Q8g9Ykmmv9ZqT
</commit_message>
<xml_diff>
--- a/KierunekZysk/2_Kierunek_Zysk_Kalkulator.xlsx
+++ b/KierunekZysk/2_Kierunek_Zysk_Kalkulator.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lejek" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dźwignie wzrostu" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Próg rentowności" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -150,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,6 +224,23 @@
     <xf numFmtId="2" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -654,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I16"/>
+  <dimension ref="B1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -778,41 +796,53 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="11" t="inlineStr"/>
-      <c r="C13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="12" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>8. Podsumowanie</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Najważniejsze liczby i diagnoza na jednym ekranie. Wyślij ten arkusz przed konsultacją Przegląd Decyzji.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="11" t="inlineStr"/>
+      <c r="C14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Kolory</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Brzoskwiniowe pola = wpisujesz. Białe pola = liczą się same (nie nadpisuj formuł).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Dane</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Wystarczą przybliżenia z faktur i kalendarza z ostatnich 12 miesięcy. Kwoty netto.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="B16" s="11" t="inlineStr">
         <is>
+          <t>Dane</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Wystarczą przybliżenia z faktur i kalendarza z ostatnich 12 miesięcy. Kwoty netto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
           <t>Licencja</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Do użytku w jednej firmie nabywcy. © guliwera4.pl</t>
         </is>
@@ -3729,4 +3759,348 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F2BFC5"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:F27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Podsumowanie: moja firma w liczbach</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Liczy się samo z pozostałych arkuszy. Wyślij przed konsultacją Przegląd Decyzji.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>Wskaźnik</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Wartość</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>Sygnał</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Co to znaczy</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Pełny koszt godziny pracy</t>
+        </is>
+      </c>
+      <c r="C6" s="47">
+        <f>Ustawienia!C12</f>
+        <v/>
+      </c>
+      <c r="D6" s="48">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="E6" s="49" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="50" t="inlineStr">
+        <is>
+          <t>Marża na klientach (z arkusza Klienci)</t>
+        </is>
+      </c>
+      <c r="C7" s="51">
+        <f>Klienci!H32</f>
+        <v/>
+      </c>
+      <c r="D7" s="52">
+        <f>IF(C7&lt;0.15,"⚠ niska",IF(C7&lt;0.3,"• średnia","✓ zdrowa"))</f>
+        <v/>
+      </c>
+      <c r="E7" s="53" t="inlineStr">
+        <is>
+          <t>Poniżej 15%: pracujecie „na obrót”</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Udział 3 największych klientów</t>
+        </is>
+      </c>
+      <c r="C8" s="34">
+        <f>Klienci!E34</f>
+        <v/>
+      </c>
+      <c r="D8" s="48">
+        <f>IF(C8&gt;0.4,"⚠ ryzyko","✓ OK")</f>
+        <v/>
+      </c>
+      <c r="E8" s="49" t="inlineStr">
+        <is>
+          <t>Powyżej 40% = ryzyko koncentracji</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="50" t="inlineStr">
+        <is>
+          <t>Klienci „Do pożegnania / wyceny” (liczba)</t>
+        </is>
+      </c>
+      <c r="C9" s="54">
+        <f>COUNTIF(Klienci!K7:K31,"*pożegnania*")</f>
+        <v/>
+      </c>
+      <c r="D9" s="52">
+        <f>IF(C9&gt;0,"⚠ do decyzji","✓ OK")</f>
+        <v/>
+      </c>
+      <c r="E9" s="53" t="inlineStr">
+        <is>
+          <t>Kandydaci do nowej wyceny lub rozstania</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Klienci „Gwiazdy” (liczba)</t>
+        </is>
+      </c>
+      <c r="C10" s="19">
+        <f>COUNTIF(Klienci!K7:K31,"⭐*")</f>
+        <v/>
+      </c>
+      <c r="D10" s="48">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="E10" s="49" t="inlineStr">
+        <is>
+          <t>Wzór idealnego klienta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="50" t="inlineStr">
+        <is>
+          <t>Najlepsza usługa (zysk na godzinę)</t>
+        </is>
+      </c>
+      <c r="C11" s="52">
+        <f>IFERROR(INDEX(Usługi!B7:B18,MATCH(1,Usługi!M7:M18,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D11" s="52">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="E11" s="53" t="inlineStr">
+        <is>
+          <t>Kandydat na usługę flagową</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Usługi ze stratą (liczba)</t>
+        </is>
+      </c>
+      <c r="C12" s="19">
+        <f>COUNTIF(Usługi!I7:I18,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="D12" s="48">
+        <f>IF(C12&gt;0,"⚠ do decyzji","✓ OK")</f>
+        <v/>
+      </c>
+      <c r="E12" s="49" t="inlineStr">
+        <is>
+          <t>Podnieś cenę, zmień zakres albo wycofaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="50" t="inlineStr">
+        <is>
+          <t>Zysk po planowanej podwyżce</t>
+        </is>
+      </c>
+      <c r="C13" s="55">
+        <f>'Podwyżka cen'!C14</f>
+        <v/>
+      </c>
+      <c r="D13" s="52">
+        <f>IF('Podwyżka cen'!C15&gt;0,"✓ +"&amp;TEXT('Podwyżka cen'!C16,"0%"),"⚠ spadek")</f>
+        <v/>
+      </c>
+      <c r="E13" s="53" t="inlineStr">
+        <is>
+          <t>Arkusz Podwyżka cen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Dopuszczalna utrata sprzedaży po podwyżce</t>
+        </is>
+      </c>
+      <c r="C14" s="34">
+        <f>'Podwyżka cen'!C17</f>
+        <v/>
+      </c>
+      <c r="D14" s="48">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="E14" s="49" t="inlineStr">
+        <is>
+          <t>Bufor bezpieczeństwa decyzji o cenach</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="50" t="inlineStr">
+        <is>
+          <t>Potrzebne zapytania / mies. (cel)</t>
+        </is>
+      </c>
+      <c r="C15" s="56">
+        <f>Lejek!D16</f>
+        <v/>
+      </c>
+      <c r="D15" s="52">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="E15" s="53" t="inlineStr">
+        <is>
+          <t>Arkusz Lejek</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Przychód potrzebny do zysku docelowego / mies.</t>
+        </is>
+      </c>
+      <c r="C16" s="36">
+        <f>'Próg rentowności'!C11</f>
+        <v/>
+      </c>
+      <c r="D16" s="48">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="E16" s="49" t="inlineStr">
+        <is>
+          <t>Arkusz Próg rentowności</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Moje 3 najważniejsze decyzje (z Dziennika decyzji)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="B19" s="57" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C19" s="58" t="n"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="B20" s="57" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C20" s="58" t="n"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="B21" s="57" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C21" s="58" t="n"/>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Decyzja, co do której mam najmniej pewności</t>
+        </is>
+      </c>
+      <c r="C23" s="58" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="59" t="inlineStr">
+        <is>
+          <t>NASTĘPNY KROK · Przegląd Decyzji (3 000 zł netto, cena pakietu odliczana). Przed spotkaniem analizuję Twoje liczby i tok rozumowania z Dziennika decyzji, a na 2-godzinnej sesji wzmacniamy najsłabsze ogniwa planu. Umów termin: guliwera4.pl/konsultacja</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="B25:E27"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C20:E20"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D6:D16">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>LEFT(D6,1)="⚠"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="4">
+      <formula>LEFT(D6,1)="✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>